<commit_message>
feat: improve API integration, listings, forms, SEO, images, and vertical branding
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\intern 2\Business-Listing\frontend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC01442-17E1-4629-B36B-32982852DCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E10E413-D7ED-40D1-AB84-4C89397521C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="93">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -67,6 +67,9 @@
     <t>Week 5</t>
   </si>
   <si>
+    <t>Dashboard / modules (if applicable to this project)</t>
+  </si>
+  <si>
     <t>Week 6</t>
   </si>
   <si>
@@ -296,15 +299,6 @@
   </si>
   <si>
     <t>Completed the Admin and User Dashboards, optimized both for responsive layouts, and completed the planned Week 6 development work. Reviewed and refined the existing frontend functionality to ensure the new dashboard components integrate correctly with the rest of the project.</t>
-  </si>
-  <si>
-    <t>Integrated and expanded the frontend functionality across authentication, dashboards, bookings, listings, products, and administration. Added Forgot Password, Reset Password, social authentication callback, Privacy, Terms, Dashboard Bookings, and Admin Settings pages. Implemented reusable components for booking requests, business products, authentication, protected routes, listing forms, and image handling. Expanded the API integration to support password reset, contact forms, social login, product management, bookings, hero image management, image uploads, owner listings and accounts, and admin management of users and listings. Enhanced the Owner Dashboard with product management, image uploads, account editing, and booking management, while updating the Admin section with functionality for users, listings, and hero images. The newly implemented features are integrated into the frontend and use demo data where the required backend functionality or data is not yet available, allowing the features to be developed and tested while the backend catches up. Also updated the project types, authentication handling, booking and review functionality, listing forms, and theme configuration.</t>
-  </si>
-  <si>
-    <t>feat: expand auth, dashboards, bookings, products, and backend integration</t>
-  </si>
-  <si>
-    <t>New frontend features and backend integrations have been implemented and connected to the project. Demo data is currently used for functionality where the corresponding backend endpoints or data are not yet available, with the structure prepared for integration once the backend implementation is completed.</t>
   </si>
 </sst>
 </file>
@@ -794,7 +788,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1">
       <c r="A1" s="13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -853,10 +847,10 @@
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F5" s="2">
         <v>5</v>
@@ -872,22 +866,22 @@
         <v>46259</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="2">
         <v>8</v>
       </c>
       <c r="G6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="198">
@@ -898,22 +892,22 @@
         <v>46260</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F7" s="2">
         <v>8</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="172.2">
@@ -924,22 +918,22 @@
         <v>46261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F8" s="2">
         <v>8</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="172.2">
@@ -950,22 +944,22 @@
         <v>46262</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F9" s="2">
         <v>8</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="159">
@@ -976,22 +970,22 @@
         <v>46264</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="2">
+        <v>8</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="2">
-        <v>8</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="184.8">
@@ -1005,19 +999,19 @@
         <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F11" s="2">
         <v>8</v>
       </c>
       <c r="G11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="184.8">
@@ -1028,22 +1022,22 @@
         <v>46266</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="2">
         <v>8</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="132">
@@ -1054,22 +1048,22 @@
         <v>46267</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F13" s="2">
         <v>8</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="118.8">
@@ -1080,22 +1074,22 @@
         <v>46268</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F14" s="2">
         <v>8</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="145.19999999999999">
@@ -1106,22 +1100,22 @@
         <v>46269</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F15" s="2">
         <v>8</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="198">
@@ -1135,19 +1129,19 @@
         <v>12</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F16" s="2">
         <v>8</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="224.4">
@@ -1158,22 +1152,22 @@
         <v>46273</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F17" s="2">
         <v>8</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="187.2">
@@ -1184,22 +1178,22 @@
         <v>46274</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F18" s="2">
         <v>8</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="105.6">
@@ -1210,22 +1204,22 @@
         <v>46275</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F19" s="2">
         <v>8</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="105.6">
@@ -1236,22 +1230,22 @@
         <v>46276</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F20" s="2">
         <v>8</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="158.4">
@@ -1265,19 +1259,19 @@
         <v>13</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F21" s="2">
         <v>8</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="224.4">
@@ -1288,22 +1282,22 @@
         <v>46280</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F22" s="2">
         <v>8</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="158.4">
@@ -1314,22 +1308,22 @@
         <v>46281</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F23" s="2">
         <v>8</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="158.4">
@@ -1337,25 +1331,25 @@
         <v>19</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F24" s="2">
         <v>8</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="237.6">
@@ -1366,49 +1360,41 @@
         <v>46283</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F25" s="2">
         <v>8</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="316.8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="2">
         <v>21</v>
       </c>
-      <c r="B26" s="5">
-        <v>46286</v>
-      </c>
+      <c r="B26" s="3"/>
       <c r="C26" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F26" s="2">
-        <v>8</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2">
@@ -1472,10 +1458,10 @@
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>10</v>
@@ -1546,10 +1532,10 @@
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>10</v>
@@ -1620,10 +1606,10 @@
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
docs: daily tracker update
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\intern 2\Business-Listing\frontend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D1BC5F4-95CE-410E-A82C-5D00864CC4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B218422-C9F2-43C6-8753-A63DF1E9943C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="129">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -433,6 +433,15 @@
   </si>
   <si>
     <t>Completed the owner notification and rider approval work on top of the latest owner dashboard changes and pushed it for review. The customer order page fixes are still to be committed. Finalized the Auto Hub website with the backend developer, and went through the SaaS gaps and fixes with the team leader.</t>
+  </si>
+  <si>
+    <t>Went through the whole SaaS restaurant project page by page in the browser (customer, owner, admin and rider pages, including phone-size screens) and made a list of the bugs and gaps for the team lead. Added a payment method popup at checkout: after pressing Place Order the customer picks Cash on Delivery, Card, Khalti or eSewa, and the options that aren't set up yet show the server's message instead of failing silently. Customers who aren't logged in are now sent to the login page before checkout. Replaced the browser's cancel order confirm box with a proper confirm dialog, and added a shared helper so popups keep focus inside them and stop the page scrolling behind. Fixed the map showing on top of popups. Fixed the customer account area: the Addresses tab could not save at all because of wrong field names, and it now has a map to pin the address; the profile shows and saves the name correctly; order history shows the restaurant and order number; and favourites show restaurant names. Moved the checkout address and map into one shared address picker used by both checkout and account. Cleaned up the new code with simplicity reviews. Merged the team lead's latest changes (auto-print on order accepted) into my branch, checked it compiles with no conflicts, and pushed it ready for a pull request. Also set up the Business Listing project in a new folder on the D drive: installed the backend and frontend packages, started a Docker Postgres database, ran all the migrations and added the starting categories.</t>
+  </si>
+  <si>
+    <t>feat(customer): payment popup, account fixes with map address picker, and order page updates</t>
+  </si>
+  <si>
+    <t>Pushed feature/customer-fixes merged with the latest main (no conflicts) and prepared the pull request for review. Listed the project's gaps for the team lead, including exposed password hashes in the delivery persons list, no automated tests, the failing production build, and the pages that still need fixing (phone layout for the owner dashboard, broken images on the owner menu, and missing admin pages). Business Listing is set up locally but still needs an admin account and the listing data imported.</t>
   </si>
 </sst>
 </file>
@@ -1822,19 +1831,31 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" ht="409.2">
       <c r="A38" s="2">
         <v>33</v>
       </c>
-      <c r="B38" s="3"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="3"/>
+      <c r="B38" s="5">
+        <v>46302</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>126</v>
+      </c>
       <c r="E38" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" s="2"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
+        <v>25</v>
+      </c>
+      <c r="F38" s="2">
+        <v>8</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="2">

</xml_diff>